<commit_message>
update daily bike stats
</commit_message>
<xml_diff>
--- a/vag-rad/vag-rad_stats.xlsx
+++ b/vag-rad/vag-rad_stats.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="723" uniqueCount="650">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="731" uniqueCount="652">
   <si>
     <t>date</t>
   </si>
@@ -1917,6 +1917,12 @@
   </si>
   <si>
     <t>2025-02-26</t>
+  </si>
+  <si>
+    <t>2025-02-27</t>
+  </si>
+  <si>
+    <t>2025-02-28</t>
   </si>
   <si>
     <t>year</t>
@@ -2328,7 +2334,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B631"/>
+  <dimension ref="A1:B633"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -7377,6 +7383,22 @@
       </c>
       <c r="B631">
         <v>1942</v>
+      </c>
+    </row>
+    <row r="632" spans="1:2">
+      <c r="A632" t="s">
+        <v>632</v>
+      </c>
+      <c r="B632">
+        <v>1889</v>
+      </c>
+    </row>
+    <row r="633" spans="1:2">
+      <c r="A633" t="s">
+        <v>633</v>
+      </c>
+      <c r="B633">
+        <v>1882</v>
       </c>
     </row>
   </sheetData>
@@ -7391,22 +7413,22 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>634</v>
+        <v>636</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>636</v>
+        <v>638</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -7414,7 +7436,7 @@
         <v>2023</v>
       </c>
       <c r="B2" t="s">
-        <v>638</v>
+        <v>640</v>
       </c>
       <c r="C2">
         <v>1793</v>
@@ -7434,7 +7456,7 @@
         <v>2023</v>
       </c>
       <c r="B3" t="s">
-        <v>639</v>
+        <v>641</v>
       </c>
       <c r="C3">
         <v>1713.5</v>
@@ -7454,7 +7476,7 @@
         <v>2023</v>
       </c>
       <c r="B4" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
       <c r="C4">
         <v>1798</v>
@@ -7474,7 +7496,7 @@
         <v>2023</v>
       </c>
       <c r="B5" t="s">
-        <v>641</v>
+        <v>643</v>
       </c>
       <c r="C5">
         <v>1810</v>
@@ -7494,7 +7516,7 @@
         <v>2023</v>
       </c>
       <c r="B6" t="s">
-        <v>642</v>
+        <v>644</v>
       </c>
       <c r="C6">
         <v>1841.5</v>
@@ -7514,7 +7536,7 @@
         <v>2023</v>
       </c>
       <c r="B7" t="s">
-        <v>643</v>
+        <v>645</v>
       </c>
       <c r="C7">
         <v>1767</v>
@@ -7534,7 +7556,7 @@
         <v>2023</v>
       </c>
       <c r="B8" t="s">
-        <v>644</v>
+        <v>646</v>
       </c>
       <c r="C8">
         <v>1785</v>
@@ -7554,7 +7576,7 @@
         <v>2023</v>
       </c>
       <c r="B9" t="s">
-        <v>645</v>
+        <v>647</v>
       </c>
       <c r="C9">
         <v>1782</v>
@@ -7574,7 +7596,7 @@
         <v>2024</v>
       </c>
       <c r="B10" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
       <c r="C10">
         <v>1708</v>
@@ -7594,7 +7616,7 @@
         <v>2024</v>
       </c>
       <c r="B11" t="s">
-        <v>647</v>
+        <v>649</v>
       </c>
       <c r="C11">
         <v>1827.5</v>
@@ -7614,7 +7636,7 @@
         <v>2024</v>
       </c>
       <c r="B12" t="s">
-        <v>648</v>
+        <v>650</v>
       </c>
       <c r="C12">
         <v>2279</v>
@@ -7634,7 +7656,7 @@
         <v>2024</v>
       </c>
       <c r="B13" t="s">
-        <v>649</v>
+        <v>651</v>
       </c>
       <c r="C13">
         <v>2011.5</v>
@@ -7654,7 +7676,7 @@
         <v>2024</v>
       </c>
       <c r="B14" t="s">
-        <v>638</v>
+        <v>640</v>
       </c>
       <c r="C14">
         <v>2315</v>
@@ -7674,7 +7696,7 @@
         <v>2024</v>
       </c>
       <c r="B15" t="s">
-        <v>639</v>
+        <v>641</v>
       </c>
       <c r="C15">
         <v>2111</v>
@@ -7694,7 +7716,7 @@
         <v>2024</v>
       </c>
       <c r="B16" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
       <c r="C16">
         <v>2068</v>
@@ -7714,7 +7736,7 @@
         <v>2024</v>
       </c>
       <c r="B17" t="s">
-        <v>641</v>
+        <v>643</v>
       </c>
       <c r="C17">
         <v>2109</v>
@@ -7734,7 +7756,7 @@
         <v>2024</v>
       </c>
       <c r="B18" t="s">
-        <v>642</v>
+        <v>644</v>
       </c>
       <c r="C18">
         <v>2031.5</v>
@@ -7754,7 +7776,7 @@
         <v>2024</v>
       </c>
       <c r="B19" t="s">
-        <v>643</v>
+        <v>645</v>
       </c>
       <c r="C19">
         <v>2040</v>
@@ -7774,7 +7796,7 @@
         <v>2024</v>
       </c>
       <c r="B20" t="s">
-        <v>644</v>
+        <v>646</v>
       </c>
       <c r="C20">
         <v>1822</v>
@@ -7794,7 +7816,7 @@
         <v>2024</v>
       </c>
       <c r="B21" t="s">
-        <v>645</v>
+        <v>647</v>
       </c>
       <c r="C21">
         <v>1893</v>
@@ -7814,7 +7836,7 @@
         <v>2025</v>
       </c>
       <c r="B22" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
       <c r="C22">
         <v>1673</v>
@@ -7834,13 +7856,13 @@
         <v>2025</v>
       </c>
       <c r="B23" t="s">
-        <v>647</v>
+        <v>649</v>
       </c>
       <c r="C23">
-        <v>1971.5</v>
+        <v>1963</v>
       </c>
       <c r="D23">
-        <v>1964.653846153846</v>
+        <v>1959</v>
       </c>
       <c r="E23">
         <v>2086</v>
@@ -7856,7 +7878,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -7961,6 +7983,22 @@
       </c>
       <c r="B13">
         <v>219</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" t="s">
+        <v>632</v>
+      </c>
+      <c r="B14">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="A15" t="s">
+        <v>633</v>
+      </c>
+      <c r="B15">
+        <v>194</v>
       </c>
     </row>
   </sheetData>
@@ -7975,22 +8013,22 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>634</v>
+        <v>636</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>636</v>
+        <v>638</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -7998,13 +8036,13 @@
         <v>2025</v>
       </c>
       <c r="B2" t="s">
-        <v>647</v>
+        <v>649</v>
       </c>
       <c r="C2">
         <v>193</v>
       </c>
       <c r="D2">
-        <v>192.4166666666666</v>
+        <v>192.1428571428572</v>
       </c>
       <c r="E2">
         <v>219</v>
@@ -8020,7 +8058,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -8125,6 +8163,22 @@
       </c>
       <c r="B13">
         <v>239</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" t="s">
+        <v>632</v>
+      </c>
+      <c r="B14">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="A15" t="s">
+        <v>633</v>
+      </c>
+      <c r="B15">
+        <v>303</v>
       </c>
     </row>
   </sheetData>
@@ -8139,22 +8193,22 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>634</v>
+        <v>636</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>636</v>
+        <v>638</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -8162,16 +8216,16 @@
         <v>2025</v>
       </c>
       <c r="B2" t="s">
-        <v>647</v>
+        <v>649</v>
       </c>
       <c r="C2">
-        <v>186</v>
+        <v>187.5</v>
       </c>
       <c r="D2">
-        <v>195.4166666666666</v>
+        <v>211.5</v>
       </c>
       <c r="E2">
-        <v>246</v>
+        <v>313</v>
       </c>
       <c r="F2">
         <v>175</v>
@@ -8184,7 +8238,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -8289,6 +8343,22 @@
       </c>
       <c r="B13">
         <v>66</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" t="s">
+        <v>632</v>
+      </c>
+      <c r="B14">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="A15" t="s">
+        <v>633</v>
+      </c>
+      <c r="B15">
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -8303,22 +8373,22 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>634</v>
+        <v>636</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>636</v>
+        <v>638</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -8326,13 +8396,13 @@
         <v>2025</v>
       </c>
       <c r="B2" t="s">
-        <v>647</v>
+        <v>649</v>
       </c>
       <c r="C2">
         <v>30</v>
       </c>
       <c r="D2">
-        <v>38.75</v>
+        <v>42.35714285714285</v>
       </c>
       <c r="E2">
         <v>68</v>

</xml_diff>